<commit_message>
added new data for PRVDRS and Dept. Just june 2026
</commit_message>
<xml_diff>
--- a/data/Departamento_de_Justicia/djDelitos.xlsx
+++ b/data/Departamento_de_Justicia/djDelitos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Departamento_de_Justicia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44749D79-680F-420F-9B98-3FCD54B29DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1B50669-B52B-47D9-B93C-6325CE1B4DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2020" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="2023" sheetId="4" r:id="rId4"/>
     <sheet name="2024" sheetId="5" r:id="rId5"/>
     <sheet name="2025" sheetId="6" r:id="rId6"/>
+    <sheet name="2026" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="30">
   <si>
     <t>FISCALIA DISTRITO</t>
   </si>
@@ -110,6 +111,24 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>TOTAL 2026</t>
+  </si>
+  <si>
+    <t>TOTAL 2025</t>
+  </si>
+  <si>
+    <t>TOTAL 2024</t>
+  </si>
+  <si>
+    <t>TOTAL 2023</t>
+  </si>
+  <si>
+    <t>TOTAL 2022</t>
+  </si>
+  <si>
+    <t>TOTAL 2021</t>
   </si>
 </sst>
 </file>
@@ -1753,7 +1772,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
@@ -2173,7 +2192,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
@@ -2593,7 +2612,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
@@ -3013,7 +3032,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
@@ -3433,7 +3452,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B15">
         <f>SUM(B2:B14)</f>
@@ -3462,6 +3481,429 @@
       <c r="H15">
         <f>SUM(B15:G15)</f>
         <v>5564</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77123BE6-D061-4C24-8876-2039ABC033E4}">
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2">
+        <v>17</v>
+      </c>
+      <c r="C2">
+        <v>125</v>
+      </c>
+      <c r="D2">
+        <v>30</v>
+      </c>
+      <c r="E2">
+        <v>58</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <f t="shared" ref="H2:H13" si="0">SUM(B2:G2)</f>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>110</v>
+      </c>
+      <c r="D3">
+        <v>25</v>
+      </c>
+      <c r="E3">
+        <v>38</v>
+      </c>
+      <c r="F3">
+        <v>4</v>
+      </c>
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <f t="shared" si="0"/>
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>74</v>
+      </c>
+      <c r="D4">
+        <v>27</v>
+      </c>
+      <c r="E4">
+        <v>35</v>
+      </c>
+      <c r="F4">
+        <v>5</v>
+      </c>
+      <c r="G4">
+        <v>4</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="0"/>
+        <v>166</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <v>169</v>
+      </c>
+      <c r="D5">
+        <v>61</v>
+      </c>
+      <c r="E5">
+        <v>76</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="0"/>
+        <v>339</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6">
+        <v>20</v>
+      </c>
+      <c r="C6">
+        <v>117</v>
+      </c>
+      <c r="D6">
+        <v>53</v>
+      </c>
+      <c r="E6">
+        <v>62</v>
+      </c>
+      <c r="F6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>3</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>260</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>15</v>
+      </c>
+      <c r="C7">
+        <v>91</v>
+      </c>
+      <c r="D7">
+        <v>22</v>
+      </c>
+      <c r="E7">
+        <v>31</v>
+      </c>
+      <c r="F7">
+        <v>4</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>163</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>111</v>
+      </c>
+      <c r="D8">
+        <v>20</v>
+      </c>
+      <c r="E8">
+        <v>57</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>93</v>
+      </c>
+      <c r="D9">
+        <v>11</v>
+      </c>
+      <c r="E9">
+        <v>30</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>87</v>
+      </c>
+      <c r="D10">
+        <v>25</v>
+      </c>
+      <c r="E10">
+        <v>42</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>174</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11">
+        <v>14</v>
+      </c>
+      <c r="C11">
+        <v>46</v>
+      </c>
+      <c r="D11">
+        <v>14</v>
+      </c>
+      <c r="E11">
+        <v>28</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12">
+        <v>38</v>
+      </c>
+      <c r="C12">
+        <v>184</v>
+      </c>
+      <c r="D12">
+        <v>44</v>
+      </c>
+      <c r="E12">
+        <v>59</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>326</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13">
+        <v>52</v>
+      </c>
+      <c r="C13">
+        <v>308</v>
+      </c>
+      <c r="D13">
+        <v>66</v>
+      </c>
+      <c r="E13">
+        <v>86</v>
+      </c>
+      <c r="F13">
+        <v>9</v>
+      </c>
+      <c r="G13">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>532</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14">
+        <v>25</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+      <c r="E14">
+        <v>10</v>
+      </c>
+      <c r="F14">
+        <v>0</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <f>SUM(B14:G14)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15">
+        <f>SUM(B2:B14)</f>
+        <v>251</v>
+      </c>
+      <c r="C15">
+        <f t="shared" ref="C15:G15" si="1">SUM(C2:C14)</f>
+        <v>1540</v>
+      </c>
+      <c r="D15">
+        <f t="shared" si="1"/>
+        <v>408</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="1"/>
+        <v>612</v>
+      </c>
+      <c r="F15">
+        <f>SUM(F2:F14)</f>
+        <v>44</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="H15">
+        <f>SUM(B15:G15)</f>
+        <v>2880</v>
       </c>
     </row>
   </sheetData>

</xml_diff>